<commit_message>
updated rule condtions test data based on review
</commit_message>
<xml_diff>
--- a/rules/CORE-000212/negative/01/data/unit-test-coreid-CG0535-negative.xlsx
+++ b/rules/CORE-000212/negative/01/data/unit-test-coreid-CG0535-negative.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanakiRaman\CORE\Rule_Authoring\core-contributor\rules\CORE-000212\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F8331A-BF1C-4F0B-9D21-5D2DD7D32FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068A22E4-361B-4DDB-8CF4-63F1D950974D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="70">
   <si>
     <t>Product</t>
   </si>
@@ -223,17 +223,23 @@
     <t>COMPLETED TREATMENT B</t>
   </si>
   <si>
-    <t>Dataset</t>
-  </si>
-  <si>
-    <t>N/A</t>
+    <t>S002</t>
+  </si>
+  <si>
+    <t>Record</t>
+  </si>
+  <si>
+    <t>DSSCAT</t>
+  </si>
+  <si>
+    <t>[ABSENT]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,8 +263,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +280,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -314,7 +331,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -332,6 +349,16 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -686,14 +713,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="23.6328125" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -713,7 +743,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -721,16 +751,237 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" t="s">
         <v>67</v>
       </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>48</v>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11">
+        <v>11</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1006,10 +1257,10 @@
       <c r="H7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="7" t="s">
         <v>57</v>
       </c>
       <c r="K7" s="4" t="s">
@@ -1032,10 +1283,10 @@
       <c r="H8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="8" t="s">
         <v>57</v>
       </c>
       <c r="K8" s="5" t="s">
@@ -1076,7 +1327,7 @@
         <v>47</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="D10">
         <v>6</v>
@@ -1084,10 +1335,10 @@
       <c r="H10" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="8" t="s">
         <v>57</v>
       </c>
       <c r="K10" s="4" t="s">
@@ -1102,7 +1353,7 @@
         <v>47</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="D11">
         <v>7</v>
@@ -1110,10 +1361,10 @@
       <c r="H11" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="8" t="s">
         <v>57</v>
       </c>
       <c r="K11" s="5" t="s">

</xml_diff>